<commit_message>
Planilha de custos: Supabase compute Small e Resend Pro como opcional
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Custos_Infra_Passaporte_de_Seguranca.xlsx
+++ b/Custos_Infra_Passaporte_de_Seguranca.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joaol\unilever-carteirinha\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FE6BF25-90E4-4DB4-B570-A8E51AE8AA29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFE19476-0E72-49D6-AB84-CE1D8932AB0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,12 +33,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="101">
   <si>
     <t>Passaporte de Segurança — Custos de Infraestrutura</t>
   </si>
   <si>
-    <t>Vercel Pro + Supabase  ·  dimensionado para ~750 usuários  ·  valores mensais recorrentes</t>
+    <t>Vercel Pro + Supabase Pro (compute Small)  ·  dimensionado para ~750 usuários  ·  valores mensais recorrentes</t>
   </si>
   <si>
     <t>Parâmetros</t>
@@ -98,10 +98,19 @@
     <t>Supabase</t>
   </si>
   <si>
-    <t>Pro</t>
-  </si>
-  <si>
-    <t>Banco Postgres, Auth (SSO), Storage e backups. Inclui US$10 de compute.</t>
+    <t>Pro (base)</t>
+  </si>
+  <si>
+    <t>Banco Postgres, Auth (SSO), Storage e backups. Inclui US$10 de crédito de compute.</t>
+  </si>
+  <si>
+    <t>Supabase — compute Small</t>
+  </si>
+  <si>
+    <t>Small</t>
+  </si>
+  <si>
+    <t>Instância Small (US$15) menos US$10 de crédito do Pro. Mais folga de CPU/memória e conexões que a Micro.</t>
   </si>
   <si>
     <t>E-mail transacional</t>
@@ -113,7 +122,7 @@
     <t>Free</t>
   </si>
   <si>
-    <t>Até 3.000 e-mails/mês grátis. Links de acesso e notificações.</t>
+    <t>Até 3.000 e-mails/mês. Para disparo em massa aos colaboradores, ver Resend Pro nos opcionais.</t>
   </si>
   <si>
     <t>Domínio / DNS</t>
@@ -143,6 +152,15 @@
     <t>Custo/mês</t>
   </si>
   <si>
+    <t>Resend Pro</t>
+  </si>
+  <si>
+    <t>50k e-mails/mês</t>
+  </si>
+  <si>
+    <t>Remove o limite de 100/dia e 3.000/mês. Necessário se for notificar os ~750 colaboradores por e-mail em massa.</t>
+  </si>
+  <si>
     <t>Assento Vercel extra</t>
   </si>
   <si>
@@ -152,13 +170,13 @@
     <t>Se mais de 1 pessoa precisar publicar/gerir deploys.</t>
   </si>
   <si>
-    <t>Supabase compute upgrade</t>
-  </si>
-  <si>
-    <t>Small/Medium</t>
-  </si>
-  <si>
-    <t>Só se o volume crescer muito. Micro já atende 750 usuários.</t>
+    <t>Supabase compute Medium</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Só se o volume crescer muito. Small já atende 750 usuários com folga.</t>
   </si>
   <si>
     <t>Domínio .com.br próprio</t>
@@ -260,7 +278,7 @@
     <t>OK</t>
   </si>
   <si>
-    <t>Conclusão: os planos Vercel Pro e Supabase Pro atendem os 750 usuários com folga. Mesmo 5.000 usuários não mudariam de tier, pois o colaborador apenas consulta (sem login) e o volume de dados é pequeno. O custo é praticamente fixo nesta escala.</t>
+    <t>Conclusão: a instância Micro já atenderia os 750 usuários. Adotamos o compute Small como margem de conforto (mais CPU, memória e conexões simultâneas), pensando em picos de acesso na troca de turno. Mesmo 5.000 usuários não mudariam de plano, pois o colaborador apenas consulta (sem login) e o volume de dados é pequeno. O custo é praticamente fixo nesta escala.</t>
   </si>
   <si>
     <t>Projeção de 12 meses</t>
@@ -923,7 +941,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:I25"/>
+  <dimension ref="B2:I27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -1047,7 +1065,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="2:9" ht="24" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:9" ht="36" x14ac:dyDescent="0.25">
       <c r="B13" s="9" t="s">
         <v>19</v>
       </c>
@@ -1075,43 +1093,43 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="2:9" ht="24" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:9" ht="36" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
         <v>23</v>
       </c>
       <c r="C14" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="10" t="s">
         <v>24</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>25</v>
       </c>
       <c r="E14" s="11">
         <v>1</v>
       </c>
       <c r="F14" s="12">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G14" s="13">
         <f>E14*F14</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H14" s="14">
         <f>G14*$C$6</f>
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I14" s="15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" ht="36" x14ac:dyDescent="0.25">
+      <c r="B15" s="9" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="15" spans="2:9" ht="24" x14ac:dyDescent="0.25">
-      <c r="B15" s="9" t="s">
+      <c r="C15" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="D15" s="10" t="s">
         <v>28</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>29</v>
       </c>
       <c r="E15" s="11">
         <v>1</v>
@@ -1128,135 +1146,146 @@
         <v>0</v>
       </c>
       <c r="I15" s="15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" ht="24" x14ac:dyDescent="0.25">
+      <c r="B16" s="9" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B16" s="16" t="s">
+      <c r="C16" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="18">
-        <f>SUM(G12:G15)</f>
-        <v>45</v>
-      </c>
-      <c r="H16" s="19">
-        <f>SUM(H12:H15)</f>
-        <v>243</v>
-      </c>
-      <c r="I16" s="17"/>
+      <c r="D16" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="E16" s="11">
+        <v>1</v>
+      </c>
+      <c r="F16" s="12">
+        <v>0</v>
+      </c>
+      <c r="G16" s="13">
+        <f>E16*F16</f>
+        <v>0</v>
+      </c>
+      <c r="H16" s="14">
+        <f>G16*$C$6</f>
+        <v>0</v>
+      </c>
+      <c r="I16" s="15" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="18">
+        <f>SUM(G12:G16)</f>
+        <v>50</v>
+      </c>
+      <c r="H17" s="19">
+        <f>SUM(H12:H16)</f>
+        <v>270</v>
+      </c>
+      <c r="I17" s="17"/>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B18" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="20">
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="20">
         <f>$C$7</f>
         <v>0.1</v>
       </c>
-      <c r="F17" s="10"/>
-      <c r="G17" s="13">
-        <f>G16*$C$7</f>
-        <v>4.5</v>
-      </c>
-      <c r="H17" s="14">
-        <f>G17*$C$6</f>
-        <v>24.3</v>
-      </c>
-      <c r="I17" s="10"/>
-    </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B18" s="21" t="s">
-        <v>32</v>
-      </c>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="23">
-        <f>G16+G17</f>
-        <v>49.5</v>
-      </c>
-      <c r="H18" s="24">
-        <f>H16+H17</f>
-        <v>267.3</v>
-      </c>
-      <c r="I18" s="22"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="13">
+        <f>G17*$C$7</f>
+        <v>5</v>
+      </c>
+      <c r="H18" s="14">
+        <f>G18*$C$6</f>
+        <v>27</v>
+      </c>
+      <c r="I18" s="10"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B19" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="26">
-        <f>G18*12</f>
-        <v>594</v>
-      </c>
-      <c r="H19" s="27">
-        <f>H18*12</f>
-        <v>3207.6000000000004</v>
-      </c>
-      <c r="I19" s="17"/>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B21" s="28" t="s">
-        <v>34</v>
-      </c>
+      <c r="B19" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="23">
+        <f>G17+G18</f>
+        <v>55</v>
+      </c>
+      <c r="H19" s="24">
+        <f>H17+H18</f>
+        <v>297</v>
+      </c>
+      <c r="I19" s="22"/>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B20" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="26">
+        <f>G19*12</f>
+        <v>660</v>
+      </c>
+      <c r="H20" s="27">
+        <f>H19*12</f>
+        <v>3564</v>
+      </c>
+      <c r="I20" s="17"/>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B22" s="29" t="s">
+      <c r="B22" s="28" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B23" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="C22" s="29" t="s">
+      <c r="C23" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="D22" s="29" t="s">
+      <c r="D23" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="G22" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="I22" s="29" t="s">
+      <c r="G23" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="I23" s="29" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="2:9" ht="24" x14ac:dyDescent="0.25">
-      <c r="B23" s="31" t="s">
-        <v>36</v>
-      </c>
-      <c r="C23" s="31" t="s">
-        <v>16</v>
-      </c>
-      <c r="D23" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="G23" s="32">
-        <v>20</v>
-      </c>
-      <c r="I23" s="15" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="24" spans="2:9" ht="24" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:9" ht="36" x14ac:dyDescent="0.25">
       <c r="B24" s="31" t="s">
         <v>39</v>
       </c>
       <c r="C24" s="31" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="D24" s="31" t="s">
         <v>40</v>
       </c>
       <c r="G24" s="32">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I24" s="15" t="s">
         <v>41</v>
@@ -1267,17 +1296,51 @@
         <v>42</v>
       </c>
       <c r="C25" s="31" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="D25" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="G25" s="33">
+      <c r="G25" s="32">
+        <v>20</v>
+      </c>
+      <c r="I25" s="15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" ht="24" x14ac:dyDescent="0.25">
+      <c r="B26" s="31" t="s">
+        <v>45</v>
+      </c>
+      <c r="C26" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="D26" s="31" t="s">
+        <v>46</v>
+      </c>
+      <c r="G26" s="32">
+        <v>60</v>
+      </c>
+      <c r="I26" s="15" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" ht="24" x14ac:dyDescent="0.25">
+      <c r="B27" s="31" t="s">
+        <v>48</v>
+      </c>
+      <c r="C27" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="D27" s="31" t="s">
+        <v>49</v>
+      </c>
+      <c r="G27" s="33">
         <f>40/12</f>
         <v>3.3333333333333335</v>
       </c>
-      <c r="I25" s="15" t="s">
-        <v>44</v>
+      <c r="I27" s="15" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1302,7 +1365,7 @@
   <sheetData>
     <row r="2" spans="2:5" ht="18" x14ac:dyDescent="0.25">
       <c r="B2" s="44" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="C2" s="41"/>
       <c r="D2" s="41"/>
@@ -1310,7 +1373,7 @@
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B3" s="40" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="C3" s="41"/>
       <c r="D3" s="41"/>
@@ -1318,119 +1381,119 @@
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B5" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="2:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B6" s="34" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="C6" s="35" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D6" s="35" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="E6" s="36" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="2:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B7" s="34" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C7" s="35" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D7" s="35" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="E7" s="36" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="2:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B8" s="34" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="C8" s="35" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="D8" s="35" t="s">
+        <v>66</v>
+      </c>
+      <c r="E8" s="36" t="s">
         <v>60</v>
-      </c>
-      <c r="E8" s="36" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="9" spans="2:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B9" s="34" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C9" s="35" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D9" s="35" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="E9" s="36" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B10" s="34" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C10" s="35" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="D10" s="35" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E10" s="36" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B11" s="34" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C11" s="35" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D11" s="35" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="E11" s="36" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B12" s="34" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="C12" s="35" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="D12" s="35" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="E12" s="36" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B14" s="43" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="C14" s="41"/>
       <c r="D14" s="41"/>
@@ -1473,7 +1536,7 @@
   <sheetData>
     <row r="2" spans="2:6" ht="18" x14ac:dyDescent="0.25">
       <c r="B2" s="44" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C2" s="41"/>
       <c r="D2" s="41"/>
@@ -1482,285 +1545,285 @@
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" s="8" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="11" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="C5" s="13">
-        <f>Custos!$G$18</f>
-        <v>49.5</v>
+        <f>Custos!$G$19</f>
+        <v>55</v>
       </c>
       <c r="D5" s="13">
         <f>C5</f>
-        <v>49.5</v>
+        <v>55</v>
       </c>
       <c r="E5" s="14">
-        <f>Custos!$H$18</f>
-        <v>267.3</v>
+        <f>Custos!$H$19</f>
+        <v>297</v>
       </c>
       <c r="F5" s="14">
         <f>E5</f>
-        <v>267.3</v>
+        <v>297</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="11" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="C6" s="13">
-        <f>Custos!$G$18</f>
-        <v>49.5</v>
+        <f>Custos!$G$19</f>
+        <v>55</v>
       </c>
       <c r="D6" s="13">
         <f t="shared" ref="D6:D16" si="0">D5+C6</f>
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="E6" s="14">
-        <f>Custos!$H$18</f>
-        <v>267.3</v>
+        <f>Custos!$H$19</f>
+        <v>297</v>
       </c>
       <c r="F6" s="14">
         <f t="shared" ref="F6:F16" si="1">F5+E6</f>
-        <v>534.6</v>
+        <v>594</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="11" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="C7" s="13">
-        <f>Custos!$G$18</f>
-        <v>49.5</v>
+        <f>Custos!$G$19</f>
+        <v>55</v>
       </c>
       <c r="D7" s="13">
         <f t="shared" si="0"/>
-        <v>148.5</v>
+        <v>165</v>
       </c>
       <c r="E7" s="14">
-        <f>Custos!$H$18</f>
-        <v>267.3</v>
+        <f>Custos!$H$19</f>
+        <v>297</v>
       </c>
       <c r="F7" s="14">
         <f t="shared" si="1"/>
-        <v>801.90000000000009</v>
+        <v>891</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="11" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="C8" s="13">
-        <f>Custos!$G$18</f>
-        <v>49.5</v>
+        <f>Custos!$G$19</f>
+        <v>55</v>
       </c>
       <c r="D8" s="13">
         <f t="shared" si="0"/>
-        <v>198</v>
+        <v>220</v>
       </c>
       <c r="E8" s="14">
-        <f>Custos!$H$18</f>
-        <v>267.3</v>
+        <f>Custos!$H$19</f>
+        <v>297</v>
       </c>
       <c r="F8" s="14">
         <f t="shared" si="1"/>
-        <v>1069.2</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" s="11" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="C9" s="13">
-        <f>Custos!$G$18</f>
-        <v>49.5</v>
+        <f>Custos!$G$19</f>
+        <v>55</v>
       </c>
       <c r="D9" s="13">
         <f t="shared" si="0"/>
-        <v>247.5</v>
+        <v>275</v>
       </c>
       <c r="E9" s="14">
-        <f>Custos!$H$18</f>
-        <v>267.3</v>
+        <f>Custos!$H$19</f>
+        <v>297</v>
       </c>
       <c r="F9" s="14">
         <f t="shared" si="1"/>
-        <v>1336.5</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="11" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="C10" s="13">
-        <f>Custos!$G$18</f>
-        <v>49.5</v>
+        <f>Custos!$G$19</f>
+        <v>55</v>
       </c>
       <c r="D10" s="13">
         <f t="shared" si="0"/>
+        <v>330</v>
+      </c>
+      <c r="E10" s="14">
+        <f>Custos!$H$19</f>
         <v>297</v>
-      </c>
-      <c r="E10" s="14">
-        <f>Custos!$H$18</f>
-        <v>267.3</v>
       </c>
       <c r="F10" s="14">
         <f t="shared" si="1"/>
-        <v>1603.8</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="11" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="C11" s="13">
-        <f>Custos!$G$18</f>
-        <v>49.5</v>
+        <f>Custos!$G$19</f>
+        <v>55</v>
       </c>
       <c r="D11" s="13">
         <f t="shared" si="0"/>
-        <v>346.5</v>
+        <v>385</v>
       </c>
       <c r="E11" s="14">
-        <f>Custos!$H$18</f>
-        <v>267.3</v>
+        <f>Custos!$H$19</f>
+        <v>297</v>
       </c>
       <c r="F11" s="14">
         <f t="shared" si="1"/>
-        <v>1871.1</v>
+        <v>2079</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" s="11" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="C12" s="13">
-        <f>Custos!$G$18</f>
-        <v>49.5</v>
+        <f>Custos!$G$19</f>
+        <v>55</v>
       </c>
       <c r="D12" s="13">
         <f t="shared" si="0"/>
-        <v>396</v>
+        <v>440</v>
       </c>
       <c r="E12" s="14">
-        <f>Custos!$H$18</f>
-        <v>267.3</v>
+        <f>Custos!$H$19</f>
+        <v>297</v>
       </c>
       <c r="F12" s="14">
         <f t="shared" si="1"/>
-        <v>2138.4</v>
+        <v>2376</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" s="11" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="C13" s="13">
-        <f>Custos!$G$18</f>
-        <v>49.5</v>
+        <f>Custos!$G$19</f>
+        <v>55</v>
       </c>
       <c r="D13" s="13">
         <f t="shared" si="0"/>
-        <v>445.5</v>
+        <v>495</v>
       </c>
       <c r="E13" s="14">
-        <f>Custos!$H$18</f>
-        <v>267.3</v>
+        <f>Custos!$H$19</f>
+        <v>297</v>
       </c>
       <c r="F13" s="14">
         <f t="shared" si="1"/>
-        <v>2405.7000000000003</v>
+        <v>2673</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14" s="11" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C14" s="13">
-        <f>Custos!$G$18</f>
-        <v>49.5</v>
+        <f>Custos!$G$19</f>
+        <v>55</v>
       </c>
       <c r="D14" s="13">
         <f t="shared" si="0"/>
-        <v>495</v>
+        <v>550</v>
       </c>
       <c r="E14" s="14">
-        <f>Custos!$H$18</f>
-        <v>267.3</v>
+        <f>Custos!$H$19</f>
+        <v>297</v>
       </c>
       <c r="F14" s="14">
         <f t="shared" si="1"/>
-        <v>2673.0000000000005</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" s="11" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C15" s="13">
-        <f>Custos!$G$18</f>
-        <v>49.5</v>
+        <f>Custos!$G$19</f>
+        <v>55</v>
       </c>
       <c r="D15" s="13">
         <f t="shared" si="0"/>
-        <v>544.5</v>
+        <v>605</v>
       </c>
       <c r="E15" s="14">
-        <f>Custos!$H$18</f>
-        <v>267.3</v>
+        <f>Custos!$H$19</f>
+        <v>297</v>
       </c>
       <c r="F15" s="14">
         <f t="shared" si="1"/>
-        <v>2940.3000000000006</v>
+        <v>3267</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" s="11" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="C16" s="13">
-        <f>Custos!$G$18</f>
-        <v>49.5</v>
+        <f>Custos!$G$19</f>
+        <v>55</v>
       </c>
       <c r="D16" s="13">
         <f t="shared" si="0"/>
-        <v>594</v>
+        <v>660</v>
       </c>
       <c r="E16" s="14">
-        <f>Custos!$H$18</f>
-        <v>267.3</v>
+        <f>Custos!$H$19</f>
+        <v>297</v>
       </c>
       <c r="F16" s="14">
         <f t="shared" si="1"/>
-        <v>3207.6000000000008</v>
+        <v>3564</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="37" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="C17" s="38">
         <f>SUM(C5:C16)</f>
-        <v>594</v>
+        <v>660</v>
       </c>
       <c r="D17" s="22"/>
       <c r="E17" s="39">
         <f>SUM(E5:E16)</f>
-        <v>3207.6000000000008</v>
+        <v>3564</v>
       </c>
       <c r="F17" s="22"/>
     </row>

</xml_diff>